<commit_message>
Monster AI phase 6 (runtime): Simple Parallel, Run Behavior, battle BT, breakpoints
- SimpleParallel composite: main task + looping background branch on a
  sub-runner sharing the Blackboard; Immediate or Delayed finish.
- RunBehavior task runs another BT with the same Blackboard (cycle and
  Blackboard checks).
- BT domain field/battle with per-task domains; battle BTs pick the
  enemy's attack each turn (UseAttack fails when the part is broken,
  UseRandomAttack = weights). Combat writes SelfHpRatio, PlayerHpRatio,
  Turn and per-part broken keys. Npcs.battle_bt column; samples
  BB_Battle and BT_Battle_Test.
- Breakpoints, pause and single step in the runner.
Test tests/test_bt_ext.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/npc.xlsx
+++ b/tools/sheets/npc.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -437,6 +437,7 @@
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -513,6 +514,11 @@
       <c r="O1" s="1" t="inlineStr">
         <is>
           <t>divinity</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>battle_bt</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1183,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>

</xml_diff>